<commit_message>
non alimentaire commentaire moins mensuel
</commit_message>
<xml_diff>
--- a/Input/redaction_template_08.xlsx
+++ b/Input/redaction_template_08.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="227">
   <si>
     <t>condition</t>
   </si>
@@ -76,9 +76,6 @@
     <t>variation_mensuelle_ipc_alim =0</t>
   </si>
   <si>
-    <t>The consumer price index experienced an increase of {evol_alim_1mois}% during the month of  {lib_mois_courant} {annee_courante} compared to the previous month.</t>
-  </si>
-  <si>
     <t>variation_mensuelle_ipc_alim* nonalim &lt; 0</t>
   </si>
   <si>
@@ -106,15 +103,6 @@
     <t>evol_non_alim_1mois=0</t>
   </si>
   <si>
-    <t xml:space="preserve"> while the consumer price index maintained the same value over a full year.</t>
-  </si>
-  <si>
-    <t>In  {lib_mois_courant} {annee_courante}, the national consumer price index maintained the same value compared to the previous month,</t>
-  </si>
-  <si>
-    <t>Over a month, the food product price index maintained the same value</t>
-  </si>
-  <si>
     <t>code</t>
   </si>
   <si>
@@ -148,24 +136,12 @@
     <t>p02_neutre</t>
   </si>
   <si>
-    <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation des ménages de la {ville} a augmenté de {evol_1mois}% par rapport au mois précédent.</t>
-  </si>
-  <si>
     <t>في شهر {lib_mois_courant } {annee_courante } ارتفعت أسعار الاستهلاك على المستوى الوطني بنسبة ({evol_1mois}% )  خلال شهر واحد</t>
   </si>
   <si>
-    <t>In  {lib_mois_courant} {annee_courante}, the national consumer price index increased by {evol_1mois}% compared to the previous month,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En glissement annuel, il a accru de {evol_12mois}%. </t>
-  </si>
-  <si>
     <t>في حين ارتفعت أسعار الاستهلاك بما يقارب  ({evol_12mois}% )  خلال سنة كاملة.</t>
   </si>
   <si>
-    <t xml:space="preserve"> while the consumer price index increased by {evol_12mois}% over a full year.</t>
-  </si>
-  <si>
     <t>p03_plus</t>
   </si>
   <si>
@@ -208,12 +184,6 @@
     <t>p06_neutre</t>
   </si>
   <si>
-    <t>the monthly variation in the non-food index increased by {evol_non_alim_1mois}% due to price increases in the following divisions: {liste_div_non_alim_plus}</t>
-  </si>
-  <si>
-    <t>The monthly variation in the non-food index stagnated following stagnation in prices in the following divisions: {liste_div_non_alim_neutre}.</t>
-  </si>
-  <si>
     <t>في حين،</t>
   </si>
   <si>
@@ -229,25 +199,16 @@
     <t>ويعزى ذلك الى زيادة أثمان {liste_pdt_alim_1mois_plus}</t>
   </si>
   <si>
-    <t>as a result of the rise in prices of {liste_pdt_alim_1mois_plus}</t>
-  </si>
-  <si>
     <t>résultat de la baisse des prix {liste_pdt_alim_1mois_moins}.</t>
   </si>
   <si>
     <t xml:space="preserve">ويعزى ذلك الى انخفاض أثمان  .{liste_pdt_alim_1mois_moins} </t>
   </si>
   <si>
-    <t>as a result of the decline in prices of {liste_pdt_alim_1mois_moins}</t>
-  </si>
-  <si>
     <t>résultat de la hausse des prix {liste_pdt_alim_1mois_plus} et de la baisse des prix {liste_pdt_alim_1mois_moins}.</t>
   </si>
   <si>
     <t>ويعزى ذلك الى زيادة أثمان {liste_pdt_alim_1mois_plus} وايضا  الى انخفاض أثمان {liste_pdt_alim_1mois_moins}</t>
-  </si>
-  <si>
-    <t>as a result of the rise in prices of {liste_pdt_alim_1mois_plus} and the decline in prices of {liste_pdt_alim_1mois_moins}</t>
   </si>
   <si>
     <t>p07_plus</t>
@@ -278,9 +239,6 @@
 العام.</t>
   </si>
   <si>
-    <t>the food product price index increased by {evol_alim_12mois}% in  {lib_mois_courant}  {annee_courante} compared to  {lib_mois_courant}  {annee_m12} , due to the rise in the prices of {liste_pdt_alim_12mois_plus}. Moreover, the decrease in prices of {liste_pdt_alim_12mois_moins} and the stagnation in prices for  {liste_pdt_alim_12mois_neutre} did not affect the general evolution.</t>
-  </si>
-  <si>
     <t>انخفض الرقم الاستدلالي للمواد الغذائية
 ب {evol_alim_12mois}% في نونبر 2025  مقارنة بنظيره من السنة الماضية،ويعزى ذلك إلى تراجع أثمان المواد المكونة للمجموعات التالية:  {liste_pdt_alim_12mois_moins}. وعلى الرغم من الارتفاعات المسجلة في أثمان المواد
 المكونة للمجموعات التالية:  {liste_pdt_alim_12mois_plus} و كذا
@@ -294,9 +252,6 @@
 الانخفاضات المسجلة في أثمان المواد المكونة للمجموعات التالية:  {liste_pdt_alim_12mois_moins} فإن ذلك لم يؤثر على التطور العام.</t>
   </si>
   <si>
-    <t>the food product price index decreased by {evol_alim_12mois}% in  {lib_mois_courant}  {annee_courante} compared to  {lib_mois_courant}  {annee_m12} , due to the decrease in the prices of {liste_pdt_alim_12mois_moins}. Moreover, the rise in prices of {liste_pdt_alim_12mois_plus} and the stagnation in prices for  {liste_pdt_alim_12mois_neutre} did not affect the general evolution.</t>
-  </si>
-  <si>
     <t>the food product price index stagnated  in  {lib_mois_courant}  {annee_courante} compared to  {lib_mois_courant}  {annee_m12} , due to the  stagnation in prices of {liste_pdt_alim_12mois_neutre}. Moreover, the rise in prices of {liste_pdt_alim_12mois_plus} and the decrease in prices of {liste_pdt_alim_12mois_moins} did not affect the general evolution.</t>
   </si>
   <si>
@@ -351,16 +306,10 @@
     <t>evol_non_alim_12mois &gt; 0</t>
   </si>
   <si>
-    <t>la variation annuelle de l'indice des produits non alimentaires a augmenté de {evol_non_alim_12mois}%.</t>
-  </si>
-  <si>
     <t>la variation annuelle de l'indice des produits non alimentaires a stagné.</t>
   </si>
   <si>
     <t>استقرالتغير السنوي لمؤشر المواد غير الغذائية ارتفاعا</t>
-  </si>
-  <si>
-    <t>the annual variation in the non-food index increased by {evol_non_alim_12mois}%.</t>
   </si>
   <si>
     <t>the annual variation in the non-food index stagnated</t>
@@ -445,9 +394,6 @@
     <t>p17</t>
   </si>
   <si>
-    <t>Indice des prix à la consommation de la {ville}: {lib_mois_courant}  {annee_courante} (base 2017: 100)</t>
-  </si>
-  <si>
     <t>Consumer price index for the {ville}: {lib_mois_courant}  {annee_courante} (2017 base: 100)</t>
   </si>
   <si>
@@ -461,18 +407,6 @@
   </si>
   <si>
     <t>على المستوى الشهري ارتفع الرقم الاستدلالي للمواد الغذائية ب {evol_alim_1mois}%  في شهر {lib_mois_courant } {annee_courante } مقارنة بشهر  .</t>
-  </si>
-  <si>
-    <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation des ménages de la {ville} a décru de {abs(evol_1mois)}% par rapport au mois précédent.</t>
-  </si>
-  <si>
-    <t>In  {lib_mois_courant} {annee_courante}, the national consumer price index decreased by {abs(evol_1mois)}% compared to the previous month,</t>
-  </si>
-  <si>
-    <t>En glissement annuel, il a décru de {abs(evol_12mois)}%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> while the consumer price index decreased by {abs(evol_12mois)}% over a full year.</t>
   </si>
   <si>
     <t>على المستوى الشهري ارتفع الرقم الاستدلالي للمواد الغذائية ب 
@@ -480,15 +414,6 @@
   في شهر {lib_mois_courant } {annee_courante } مقارنة بشهر  {lib_mois_m1 } .{annee_m1 }</t>
   </si>
   <si>
-    <t>The consumer price index experienced a decrease of {abs(evol_alim_1mois)}% during the month of  {lib_mois_courant} {annee_courante} compared to the previous month.</t>
-  </si>
-  <si>
-    <t>la variation annuelle de l'indice des produits non alimentaires a diminué de {abs(evol_non_alim_12mois)}%.</t>
-  </si>
-  <si>
-    <t>the annual variation in the non-food index decreased by {abs(evol_non_alim_12mois)}%.</t>
-  </si>
-  <si>
     <t>في حين انخفضت أسعار الاستهلاك بما يقارب  ({abs(evol_12mois)}'% )  خلال سنة كاملة.</t>
   </si>
   <si>
@@ -498,95 +423,7 @@
     <t>سجل التغير السنوي لمؤشر المواد غير الغذائية انخفاضا ب {abs(evol_non_alim_12mois)}'%،</t>
   </si>
   <si>
-    <r>
-      <t>l'indice des prix des produits alimentaires a</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> augmenté</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> de {evol_alim_1mois}% en {lib_mois_courant} {annee_courante} par rapport à  {lib_mois_m1} {annee_m1},</t>
-    </r>
-  </si>
-  <si>
-    <t>l'indice des prix des produits alimentaires a diminué de {abs(evol_alim_1mois)}% en {lib_mois_courant} {annee_courante} par rapport à  {lib_mois_m1} {annee_m1},</t>
-  </si>
-  <si>
-    <t>l'indice des prix des produits alimentaires a maintenu la même évolution en {lib_mois_courant} {annee_courante} par rapport à  {lib_mois_m1} {annee_m1},</t>
-  </si>
-  <si>
     <t>كما،</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">la variation mensuelle de l'indice des produits non alimentaires a accru de  {evol_non_alim_1mois}% en raison de la hausse des prix des divisions suivantes: {liste_div_non_alim_plus}. Aussi la baisse des prix </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">des divisions suivantes : </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>{liste_div_non_alim_moins}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Ainsi que,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> la stagnation des indices des autres
-divisions n’ont pas impacté l'évolution générale.</t>
-    </r>
-  </si>
-  <si>
-    <t>l’indice des prix des produits alimentaires
-a accru de {evol_alim_12mois}% en {lib_mois_courant} {annee_courante} par rapport à {lib_mois_courant} {annee_m12}, sous l'effet de l’augmentation des
-prix  {liste_pdt_alim_12mois_plus}. Par ailleurs, la diminution des prix {liste_pdt_alim_12mois_moins} et la stagnation des prix  {liste_pdt_alim_12mois_neutre} n’ont pas affecté l’évolution
-générale.</t>
-  </si>
-  <si>
-    <t>l’indice des prix des produits alimentaires
-a baissé de {evol_alim_12mois}% en {lib_mois_courant} {annee_courante} par rapport à {lib_mois_courant} {annee_m12}, sous l'effet de la diminution des
-prix  {liste_pdt_alim_12mois_moins}. Par ailleurs, l'augmentation des prix {liste_pdt_alim_12mois_plus} et la stagnation des prix  {liste_pdt_alim_12mois_neutre} n’ont pas affecté l’évolution générale.</t>
   </si>
   <si>
     <t>l’indice des prix des produits alimentaires
@@ -597,9 +434,6 @@
     <t>p13_0</t>
   </si>
   <si>
-    <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a augmenté de {evol_12mois}% par rapport à {lib_mois_courant} {annee_m12}</t>
-  </si>
-  <si>
     <t xml:space="preserve">في {lib_mois_courant } {annee_courante } ارتفع الرقم الاستدلالي للأثمان عند الاستهلاك
 ب {evol_12mois} % مقارنة بشهر {lib_mois_courant } {annee_m12 } </t>
   </si>
@@ -607,22 +441,13 @@
     <t xml:space="preserve">قراءة: </t>
   </si>
   <si>
-    <t>In {lib_mois_courant} {annee_courante}, the consumer price index increased by {evol_12mois}% compared to {lib_mois_courant} {annee_m12}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reading: </t>
-  </si>
-  <si>
-    <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a décru de {abs(evol_12mois)}% par rapport à {lib_mois_courant} {annee_m12}</t>
   </si>
   <si>
     <t xml:space="preserve">في {lib_mois_courant } {annee_courante } انخفض الرقم الاستدلالي للأثمان عند الاستهلاك
 {abs(evol_12mois)}'% مقارنة بشهر {lib_mois_courant } {annee_m12 } </t>
   </si>
   <si>
-    <t>In {lib_mois_courant} {annee_courante}, the consumer price index decreased by {abs(evol_12mois)}% compared to {lib_mois_courant} {annee_m12}</t>
-  </si>
-  <si>
     <t>In {lib_mois_courant} {annee_courante}, the consumer price index decreased stagnated compared to {lib_mois_courant} {annee_m12}</t>
   </si>
   <si>
@@ -634,12 +459,6 @@
 ب {evol_1mois} % مقارنة بشهر {lib_mois_m1} {annee_m1 } </t>
   </si>
   <si>
-    <t>In {lib_mois_courant} {annee_courante}, the consumer price index increased by {evol_1mois}% compared to {lib_mois_m1} {annee_m1}</t>
-  </si>
-  <si>
-    <t>In {lib_mois_courant} {annee_courante}, the consumer price index decreased stagnated compared to {lib_mois_m1} {annee_m1}</t>
-  </si>
-  <si>
     <t>p20_0</t>
   </si>
   <si>
@@ -667,65 +486,128 @@
     <t xml:space="preserve">Lecture: </t>
   </si>
   <si>
-    <t>Alors que la variation des prix des divisions qui constituent les produits non alimentaires a fluctué entre une diminution de la division {liste_min_div_non_alim_12mois_moins} et une augmentation de la division {liste_max_div_non_alim_12mois_plus}</t>
-  </si>
-  <si>
-    <r>
-      <t>la variation mensuelle de l'indice des produits non alimentaires a décru de  {abs(evol_non_alim_1mois)}% en raison de la baisse des prix des divisions suivantes: {liste_div_non_alim_moins}. Aussi la hausse hausse des prix {liste_div_non_alim_plus}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Ainsi que,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> la stagnation des indices des autres
-divisions n’ont pas impacté l'évolution générale.</t>
-    </r>
-  </si>
-  <si>
     <t>انخفض التغير الشهري للرقم الاستدلالي للمواد غير الغذائية ب  ( abs(evol_non_alim_1mois) % ) جراء انخفاض أثمان الأقسام التالية: {liste_div_non_alim_moins} .</t>
-  </si>
-  <si>
-    <t>the monthly variation in the non-food index decreased by abs(evol_non_alim_1mois)% due to price decreases in the following divisions: {liste_div_non_alim_moins}.</t>
   </si>
   <si>
     <t xml:space="preserve">في {lib_mois_courant } {annee_courante } انخفظ الرقم الاستدلالي للأثمان عند الاستهلاك
 ب {abs(evol_1mois)} % مقارنة بشهر {lib_mois_m1} {annee_m1 } </t>
   </si>
   <si>
-    <t>In {lib_mois_courant} {annee_courante}, the consumer price index decreased by {abs(evol_1mois)}% compared to {lib_mois_m1} {annee_m1}</t>
+    <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation des ménages de la {ville} a augmenté de {fmt(evol_1mois)}% par rapport au mois précédent.</t>
+  </si>
+  <si>
+    <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation des ménages de la {ville} a décru de {fmt(abs(evol_1mois))}% par rapport au mois précédent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En glissement annuel, il a accru de {fmt(evol_12mois)}%. </t>
+  </si>
+  <si>
+    <t>En glissement annuel, il a décru de {fmt(abs(evol_12mois))}%.</t>
+  </si>
+  <si>
+    <t>l'indice des prix des produits alimentaires a diminué de {fmt(abs(evol_alim_1mois))}% en {lib_mois_courant} {annee_courante} par rapport à  {lib_mois_m1} {annee_m1},</t>
+  </si>
+  <si>
+    <t>l’indice des prix des produits alimentaires
+a accru de {fmt(evol_alim_12mois)}% en {lib_mois_courant} {annee_courante} par rapport à {lib_mois_courant} {annee_m12}, sous l'effet de l’augmentation des
+prix  {liste_pdt_alim_12mois_plus}. Par ailleurs, la diminution des prix {liste_pdt_alim_12mois_moins} et la stagnation des prix  {liste_pdt_alim_12mois_neutre} n’ont pas affecté l’évolution
+générale.</t>
+  </si>
+  <si>
+    <t>la variation annuelle de l'indice des produits non alimentaires a augmenté de {fmt(evol_non_alim_12mois)}%.</t>
+  </si>
+  <si>
+    <t>la variation annuelle de l'indice des produits non alimentaires a diminué de {fmt(abs(evol_non_alim_12mois))}%.</t>
+  </si>
+  <si>
+    <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a augmenté de {fmt(evol_12mois)}% par rapport à {lib_mois_courant} {annee_m12}</t>
+  </si>
+  <si>
+    <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a décru de {fmt(abs(evol_12mois))}% par rapport à {lib_mois_courant} {annee_m12}</t>
+  </si>
+  <si>
+    <t>Alors que la variation des prix des divisions qui constituent les produits non alimentaires a fluctué entre une diminution {liste_min_div_non_alim_12mois_moins} et une augmentation  {liste_max_div_non_alim_12mois_plus}</t>
+  </si>
+  <si>
+    <t>In  {lib_mois_courant} {annee_courante}, the national consumer price index maintained the same value compared to the previous month.</t>
+  </si>
+  <si>
+    <t>In  {lib_mois_courant} {annee_courante}, the consumer price index for households increased by {fmt(evol_1mois)}% compared to the previous month.</t>
+  </si>
+  <si>
+    <t>On an annual level, the consumer price index increased by {fmt(evol_12mois)}% over a full year.</t>
+  </si>
+  <si>
+    <t>On an annual level, the consumer price index decreased by {fmt(abs(evol_12mois))}% over a full year.</t>
+  </si>
+  <si>
+    <t>On an annual level, the consumer price index maintained the same value over a full year.</t>
+  </si>
+  <si>
+    <t>l'indice des prix des produits alimentaires a augmenté de {fmt(evol_alim_1mois)}% en {lib_mois_courant} {annee_courante} par rapport à  {lib_mois_m1} {annee_m1},</t>
+  </si>
+  <si>
+    <t>as a result of the rise in prices of {liste_pdt_alim_1mois_plus}.</t>
+  </si>
+  <si>
+    <t>as a result of the decline in prices of {liste_pdt_alim_1mois_moins}.</t>
+  </si>
+  <si>
+    <t>as a result of the rise in prices of {liste_pdt_alim_1mois_plus} and the decline in prices of {liste_pdt_alim_1mois_moins}.</t>
+  </si>
+  <si>
+    <t>In  {lib_mois_courant} {annee_courante}, the consumer price index for households decreased by {fmt(evol_1mois)}% compared to the previous month.</t>
+  </si>
+  <si>
+    <t>the food price index remained unchanged in  {lib_mois_courant} {annee_courante} compared to {lib_mois_m1} {annee_m1}.</t>
+  </si>
+  <si>
+    <t>l'indice des prix des produits alimentaires a maintenu la même évolution en {lib_mois_courant} {annee_courante} par rapport à  {lib_mois_m1} {annee_m1}.</t>
+  </si>
+  <si>
+    <t>Moreover,</t>
+  </si>
+  <si>
+    <t>the monthly variation of the index for the non-food products increased by {fmt(evol_non_alim_1mois)}% due to the increase in prices  in the following divisions: {liste_div_non_alim_plus}. Also, the decrease in prices of the following divisions: {liste_div_non_alim_moins}. Thus, the stagnation of the indices of the other divisions did not impact the general evolution.</t>
+  </si>
+  <si>
+    <t>the monthly variation of the index for the non-food products decreased by {fmt(abs(evol_non_alim_1mois))}% due to drop in prices in the following divisions: {liste_div_non_alim_moins}. Also, the increase in prices of the following divisions: {liste_div_non_alim_plus}. Thus, the stagnation of the indices of the other divisions did not impact the general evolution.</t>
+  </si>
+  <si>
+    <t>The monthly variation of the index for the non-food products stagnated following stagnation in prices in the following divisions: {liste_div_non_alim_neutre}.Also, the increase in prices of the following divisions: {liste_div_non_alim_plus} and the decrease in prices of the following divisions: {liste_div_non_alim_moins},  did not impact the general evolution.</t>
+  </si>
+  <si>
+    <t>The food product price index increased by {fmt(evol_alim_1mois)}% in  {lib_mois_courant} {annee_courante} compared to {lib_mois_m1} {annee_m1},</t>
+  </si>
+  <si>
+    <t>The  food product price index decreased by {fmt(abs(evol_alim_1mois))}% in  {lib_mois_courant} {annee_courante} compared to {lib_mois_m1} {annee_m1},</t>
+  </si>
+  <si>
+    <t>the food product price index increased by {fmt(evol_alim_12mois)}% in  {lib_mois_courant}  {annee_courante} compared to  {lib_mois_courant}  {annee_m12} , due to the rise in the prices of {liste_pdt_alim_12mois_plus}. Moreover, the decrease in prices of {liste_pdt_alim_12mois_moins} and the stagnation in prices for  {liste_pdt_alim_12mois_neutre} did not affect the general evolution.</t>
+  </si>
+  <si>
+    <t>l’indice des prix des produits alimentaires
+a baissé de {fmt(abs(evol_alim_12mois))}% en {lib_mois_courant} {annee_courante} par rapport à {lib_mois_courant} {annee_m12}, sous l'effet de la diminution des
+prix  {liste_pdt_alim_12mois_moins}. Par ailleurs, l'augmentation des prix {liste_pdt_alim_12mois_plus} et la stagnation des prix  {liste_pdt_alim_12mois_neutre} n’ont pas affecté l’évolution générale.</t>
+  </si>
+  <si>
+    <t>the food product price index decreased by {fmt(abs(evol_alim_12mois))}% in  {lib_mois_courant}  {annee_courante} compared to  {lib_mois_courant}  {annee_m12} , due to the decrease in the prices of {liste_pdt_alim_12mois_moins}. Moreover, the rise in prices of {liste_pdt_alim_12mois_plus} and the stagnation in prices for  {liste_pdt_alim_12mois_neutre} did not affect the general evolution.</t>
+  </si>
+  <si>
+    <t>the annual variation in the non-food index increased by {fmt(evol_non_alim_12mois)}%.</t>
+  </si>
+  <si>
+    <t>the annual variation in the non-food index decreased by {fmt(abs(evol_non_alim_12mois))}%.</t>
+  </si>
+  <si>
+    <t>In {lib_mois_courant} {annee_courante}, the consumer price index increased by {fmt(evol_12mois)}% compared to {lib_mois_courant} {annee_m12}</t>
+  </si>
+  <si>
+    <t>In {lib_mois_courant} {annee_courante}, the consumer price index decreased by {fmt(abs(evol_12mois))}% compared to {lib_mois_courant} {annee_m12}</t>
   </si>
   <si>
     <r>
-      <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a augmenté de {evol_1mois}% par rapport</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> {lib_mois_m1} {annee_m1}</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a gardé la même valeur</t>
+      <t>La variation des prix en {lib_mois_courant} {annee_courante}, a gardé la même valeur</t>
     </r>
     <r>
       <rPr>
@@ -744,11 +626,128 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>par rapport à {lib_mois_m1} {annee_m1}</t>
+      <t xml:space="preserve"> après avoir  été {fmt(evol_mois1_mois1)}% en {lib_mois_m2} {annee_m1}</t>
     </r>
   </si>
   <si>
-    <t>En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a diminué de {abs(evol_1mois)}% par rapport à {lib_mois_m1} {annee_m1}</t>
+    <t>La variation des prix en {lib_mois_courant} {annee_courante}, a diminué de {fmt(abs(evol_1mois))}%  après avoir  été de {fmt(evol_mois1_mois2)}% en {lib_mois_m1} {annee_m1}</t>
+  </si>
+  <si>
+    <t>La variation des prix en {lib_mois_courant} {annee_courante} a augmenté de {fmt(evol_1mois)}% après avoir  été de {fmt(evol_mois1_mois2)}% en {lib_mois_m1} {annee_m1}</t>
+  </si>
+  <si>
+    <t>The level of price variation in {lib_mois_courant} {annee_courante} increased by  {fmt(abs(evol_1mois))}% after being {fmt(evol_mois1_mois2)}% in {lib_mois_m2} {annee_m2}</t>
+  </si>
+  <si>
+    <t>The level of price variation in {lib_mois_courant} {annee_courante} decreased by  {fmt(abs(evol_1mois))}% after being {fmt(evol_mois1_mois2)}% in {lib_mois_m2} {annee_m2}</t>
+  </si>
+  <si>
+    <t>In {lib_mois_courant} {annee_courante}, the consumer price index stagnated after being {fmt(evol_mois1_mois2)}% in {lib_mois_m1} {annee_m1}</t>
+  </si>
+  <si>
+    <t>Indice des prix à la consommation de la {ville}: {lib_mois_courant_prep}  {annee_courante} (base 2017: 100)</t>
+  </si>
+  <si>
+    <t>p06_plus_moins_1</t>
+  </si>
+  <si>
+    <t>la variation mensuelle de l'indice des produits non alimentaires a accru de  {fmt(evol_non_alim_1mois)}% en raison de la hausse des prix des divisions suivantes: {liste_div_non_alim_plus}.</t>
+  </si>
+  <si>
+    <t>p06_plus_moins</t>
+  </si>
+  <si>
+    <t>evol_non_alim_1mois&gt;1</t>
+  </si>
+  <si>
+    <t>la baisse des prix des divisions suivantes: {liste_div_non_alim_moins}.</t>
+  </si>
+  <si>
+    <t>p06_plus_neutre</t>
+  </si>
+  <si>
+    <t>p06_plus_neutre_1</t>
+  </si>
+  <si>
+    <t>p06_plus_neutre_prep</t>
+  </si>
+  <si>
+    <t>evol_non_alim_1mois&gt;2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ainsi que, </t>
+  </si>
+  <si>
+    <t>la stagnation des indices de la division {liste_div_non_alim_neutre}</t>
+  </si>
+  <si>
+    <t>p06_plus_moins_prep</t>
+  </si>
+  <si>
+    <t>p06_plus_fin</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> n’ont pas impacté l'évolution générale.</t>
+  </si>
+  <si>
+    <t>p06_plus_fin_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> n’a pas impacté l'évolution générale.</t>
+  </si>
+  <si>
+    <t>p06_plus_1</t>
+  </si>
+  <si>
+    <t>la variation mensuelle de l'indice des produits non alimentaires a accru de  {fmt(evol_non_alim_1mois)}% en raison de la hausse des prix de la division suivante: {liste_div_non_alim_plus}.</t>
+  </si>
+  <si>
+    <t>la baisse des prix de la division: {liste_div_non_alim_moins}.</t>
+  </si>
+  <si>
+    <t>p06_moins_1</t>
+  </si>
+  <si>
+    <t>la variation mensuelle de l'indice des produits non alimentaires a décru de  {fmt(abs(evol_non_alim_1mois))}% en raison de la baisse des prix de la division suivante: {liste_div_non_alim_moins}</t>
+  </si>
+  <si>
+    <t>p06_moins_plus_prep</t>
+  </si>
+  <si>
+    <t>p06_moins_plus</t>
+  </si>
+  <si>
+    <t>la hausse des prix des divisions suivantes: {liste_div_non_alim_plus}.</t>
+  </si>
+  <si>
+    <t>la hausse des prix des division suivante: {liste_div_non_alim_plus}.</t>
+  </si>
+  <si>
+    <t>p06_moins_plus_1</t>
+  </si>
+  <si>
+    <t>p06_moins_neutre_prep</t>
+  </si>
+  <si>
+    <t>p06_moins_neutre</t>
+  </si>
+  <si>
+    <t>p06_moins_neutre_1</t>
+  </si>
+  <si>
+    <t>la stagnation des indices des autres divisions</t>
+  </si>
+  <si>
+    <t>p06_moins_fin</t>
+  </si>
+  <si>
+    <t>p06_moins_fin_1</t>
+  </si>
+  <si>
+    <t>la variation mensuelle de l'indice des produits non alimentaires a décru de  {fmt(abs(evol_non_alim_1mois))}% en raison de la baisse des prix des divisions suivantes: {liste_div_non_alim_moins}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aussi, </t>
   </si>
 </sst>
 </file>
@@ -821,7 +820,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -834,6 +833,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1116,7 +1118,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="1"/>
@@ -1130,7 +1132,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1150,50 +1152,50 @@
     </row>
     <row r="2" spans="1:6" ht="45">
       <c r="A2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>42</v>
+        <v>150</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>44</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="45">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>144</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="45">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>9</v>
@@ -1205,55 +1207,55 @@
         <v>11</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>29</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30">
       <c r="A5" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>45</v>
+        <v>152</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>47</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>151</v>
+        <v>126</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>12</v>
@@ -1265,648 +1267,963 @@
         <v>14</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>28</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="60">
       <c r="A8" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>154</v>
+      <c r="D8" s="6" t="s">
+        <v>166</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="60">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="45">
       <c r="A9" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>182</v>
+        <v>145</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="45">
       <c r="A10" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>124</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="30">
       <c r="A11" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>69</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="30">
       <c r="A12" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>72</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="45">
       <c r="A13" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>75</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="30">
       <c r="A14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="30">
       <c r="A15" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>157</v>
+        <v>129</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="30">
       <c r="A16" s="1" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="105">
       <c r="A17" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>62</v>
+        <v>174</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="105">
       <c r="A18" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>60</v>
+        <v>209</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>187</v>
+        <v>56</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="90">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>61</v>
+        <v>204</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>27</v>
+        <v>196</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="135">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="30">
       <c r="A20" s="1" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>76</v>
+        <v>195</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>77</v>
+        <v>196</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="120">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>78</v>
+        <v>193</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>81</v>
+        <v>196</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="120">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>79</v>
+        <v>200</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>82</v>
+        <v>201</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="30">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="105">
       <c r="A23" s="1" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>90</v>
+        <v>198</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>94</v>
+        <v>222</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="105">
       <c r="A24" s="1" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>91</v>
+        <v>199</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>96</v>
+        <v>203</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>56</v>
       </c>
       <c r="F24" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="105">
+      <c r="A25" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="30">
+      <c r="D25" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="105">
       <c r="A26" s="1" t="s">
-        <v>99</v>
+        <v>47</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>100</v>
+        <v>207</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>105</v>
+        <v>24</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>111</v>
+        <v>208</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>56</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="30">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="105">
       <c r="A27" s="1" t="s">
-        <v>99</v>
+        <v>47</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>153</v>
+        <v>225</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="30">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="105">
       <c r="A28" s="1" t="s">
-        <v>99</v>
+        <v>47</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>102</v>
+        <v>212</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>103</v>
+        <v>25</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>108</v>
+        <v>213</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>56</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="75">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29" s="1" t="s">
-        <v>112</v>
+        <v>47</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>112</v>
+        <v>214</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>113</v>
+        <v>226</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="30">
       <c r="A30" s="1" t="s">
-        <v>115</v>
+        <v>47</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>115</v>
+        <v>215</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="30">
       <c r="A31" s="1" t="s">
-        <v>162</v>
+        <v>47</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>162</v>
+        <v>218</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="45">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32" s="1" t="s">
-        <v>116</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>117</v>
+        <v>219</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>133</v>
+        <v>25</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="45">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="105">
       <c r="A33" s="1" t="s">
-        <v>116</v>
+        <v>47</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>118</v>
+        <v>220</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>134</v>
+        <v>25</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>168</v>
+        <v>222</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>169</v>
+        <v>56</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="45">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="105">
       <c r="A34" s="1" t="s">
-        <v>116</v>
+        <v>47</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>119</v>
+        <v>221</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>172</v>
+        <v>56</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="30">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="105">
       <c r="A35" s="1" t="s">
-        <v>120</v>
+        <v>47</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>120</v>
+        <v>223</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>124</v>
+        <v>206</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>122</v>
+        <v>56</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="45">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="105">
       <c r="A36" s="1" t="s">
-        <v>125</v>
+        <v>47</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>128</v>
+        <v>224</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>130</v>
+        <v>25</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>191</v>
+        <v>208</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>173</v>
+        <v>56</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="45">
+    <row r="37" spans="1:6" ht="105">
       <c r="A37" s="1" t="s">
-        <v>125</v>
+        <v>47</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>127</v>
+        <v>53</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>129</v>
+        <v>26</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>193</v>
+        <v>123</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>189</v>
+        <v>55</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="45">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="135">
       <c r="A38" s="1" t="s">
-        <v>125</v>
+        <v>67</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>126</v>
+        <v>63</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>131</v>
+        <v>64</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>192</v>
+        <v>155</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>132</v>
+        <v>70</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="30">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="135">
       <c r="A39" s="1" t="s">
-        <v>136</v>
+        <v>67</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>136</v>
+        <v>65</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>139</v>
+        <v>71</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="120">
       <c r="A40" s="1" t="s">
-        <v>176</v>
+        <v>67</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>176</v>
+        <v>66</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>178</v>
+        <v>130</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>180</v>
+        <v>72</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>178</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="30">
       <c r="A41" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="30">
+      <c r="A44" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="30">
+      <c r="A45" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="30">
+      <c r="A46" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="75">
+      <c r="A47" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="30">
+      <c r="A48" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="45">
+      <c r="A50" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="45">
+      <c r="A51" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="45">
+      <c r="A52" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="30">
+      <c r="A53" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="60">
+      <c r="A54" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="60">
+      <c r="A55" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="45">
+      <c r="A56" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="30">
+      <c r="A57" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="30">
+      <c r="A59" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D59" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>181</v>
+      <c r="E59" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
version fr et ang ok
</commit_message>
<xml_diff>
--- a/Input/redaction_template_08.xlsx
+++ b/Input/redaction_template_08.xlsx
@@ -776,9 +776,6 @@
     <t>La variation mensuelle de l'indice des produits non alimentaires a stagné suite à la stagnation des prix de la division: {liste_div_non_alim_neutre}.</t>
   </si>
   <si>
-    <t>In  {lib_mois_courant} {annee_courante},  the consumer price index for households in the city of {ville} maintained the same value compared to the previous month.</t>
-  </si>
-  <si>
     <t>the food price index remained unchanged in  {lib_mois_courant} {annee_courante} compared to {lib_mois_m1} {annee_m1},</t>
   </si>
   <si>
@@ -812,9 +809,6 @@
     <t>the monthly variation of the index for the non-food products index increased by {fmt(evol_non_alim_1mois)}% due to the increase in prices  in the following divisions: {liste_div_non_alim_plus}.</t>
   </si>
   <si>
-    <t xml:space="preserve">the monthly variation of the index for the non-food products increased by {fmt(evol_non_alim_1mois)}% due to the increase in prices of: {liste_div_non_alim_plus}. </t>
-  </si>
-  <si>
     <t>the increase in prices of the following divisions: {liste_div_non_alim_plus}.</t>
   </si>
   <si>
@@ -879,9 +873,6 @@
   </si>
   <si>
     <t>the annual variation in the non-food product index increased by {fmt(evol_non_alim_12mois)}%.</t>
-  </si>
-  <si>
-    <t>Evolution of the monthly variation of the consumer price index</t>
   </si>
   <si>
     <t>The level of price variation in {lib_mois_courant} {annee_courante} increased by  {fmt(evol_1mois)}% after being {fmt(evol_mois1_mois2)}% in {lib_mois_m1} {annee_m1}</t>
@@ -920,9 +911,6 @@
     <t>In  {lib_mois_courant} {annee_courante}, the consumer price index for households in the {ville} increased by {fmt(evol_1mois)}% compared to the previous month.</t>
   </si>
   <si>
-    <t>In  {lib_mois_courant} {annee_courante}, the consumer price index for households in the city of {ville} decreased by {fmt(abs(evol_1mois))}% compared to the previous month.</t>
-  </si>
-  <si>
     <t>On an annual level, the consumer price index increased by {fmt(evol_12mois)}%.</t>
   </si>
   <si>
@@ -945,6 +933,18 @@
   </si>
   <si>
     <t>The level of price variation in {lib_mois_courant} {annee_courante} decreased by  {fmt(abs(evol_1mois))}% after being {fmt(evol_mois1_mois2)}% in {lib_mois_m1} {annee_m2}</t>
+  </si>
+  <si>
+    <t>In  {lib_mois_courant} {annee_courante}, the consumer price index for households in the {ville} decreased by {fmt(abs(evol_1mois))}% compared to the previous month.</t>
+  </si>
+  <si>
+    <t>In  {lib_mois_courant} {annee_courante},  the consumer price index for households in the {ville} maintained the same value compared to the previous month.</t>
+  </si>
+  <si>
+    <t>the monthly variation of the index for the non-food products decreased by {fmt(abs(evol_non_alim_1mois))}% due to the decrease in prices of: {liste_div_non_alim_moins}.</t>
+  </si>
+  <si>
+    <t>Evolution of the monthly variation (%) of the consumer price index</t>
   </si>
 </sst>
 </file>
@@ -1316,7 +1316,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1373,7 +1373,7 @@
         <v>38</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="45">
@@ -1393,7 +1393,7 @@
         <v>122</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="45">
@@ -1413,7 +1413,7 @@
         <v>11</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>243</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30">
@@ -1433,7 +1433,7 @@
         <v>39</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30">
@@ -1453,7 +1453,7 @@
         <v>121</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30">
@@ -1473,7 +1473,7 @@
         <v>14</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="60">
@@ -1533,7 +1533,7 @@
         <v>119</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1553,7 +1553,7 @@
         <v>58</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1573,7 +1573,7 @@
         <v>60</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="45">
@@ -1673,7 +1673,7 @@
         <v>56</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="60">
@@ -1693,7 +1693,7 @@
         <v>56</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1710,7 +1710,7 @@
         <v>195</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="30">
@@ -1727,7 +1727,7 @@
         <v>169</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1744,7 +1744,7 @@
         <v>182</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1761,7 +1761,7 @@
         <v>174</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="45">
@@ -1781,7 +1781,7 @@
         <v>56</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="45">
@@ -1801,7 +1801,7 @@
         <v>56</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="45">
@@ -1821,7 +1821,7 @@
         <v>56</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="45">
@@ -1841,7 +1841,7 @@
         <v>56</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="60">
@@ -1861,7 +1861,7 @@
         <v>142</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="60">
@@ -1881,7 +1881,7 @@
         <v>56</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>255</v>
+        <v>291</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1898,7 +1898,7 @@
         <v>195</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="30">
@@ -1915,7 +1915,7 @@
         <v>186</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="30">
@@ -1932,7 +1932,7 @@
         <v>241</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1949,7 +1949,7 @@
         <v>174</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="45">
@@ -1969,7 +1969,7 @@
         <v>56</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="45">
@@ -1989,7 +1989,7 @@
         <v>56</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="45">
@@ -2009,7 +2009,7 @@
         <v>56</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="45">
@@ -2029,7 +2029,7 @@
         <v>56</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="45">
@@ -2049,7 +2049,7 @@
         <v>55</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="45">
@@ -2069,7 +2069,7 @@
         <v>56</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -2086,7 +2086,7 @@
         <v>195</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="40" spans="1:6" s="7" customFormat="1" ht="30">
@@ -2103,7 +2103,7 @@
         <v>200</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="41" spans="1:6" s="7" customFormat="1">
@@ -2120,7 +2120,7 @@
         <v>202</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="42" spans="1:6" s="7" customFormat="1">
@@ -2137,7 +2137,7 @@
         <v>204</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="43" spans="1:6" s="7" customFormat="1" ht="45">
@@ -2157,7 +2157,7 @@
         <v>56</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="44" spans="1:6" s="7" customFormat="1" ht="45">
@@ -2177,7 +2177,7 @@
         <v>56</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="45" spans="1:6" s="7" customFormat="1" ht="45">
@@ -2197,7 +2197,7 @@
         <v>56</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="45">
@@ -2217,7 +2217,7 @@
         <v>56</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="120">
@@ -2237,7 +2237,7 @@
         <v>70</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="120">
@@ -2277,7 +2277,7 @@
         <v>70</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="120">
@@ -2297,7 +2297,7 @@
         <v>70</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="120">
@@ -2317,7 +2317,7 @@
         <v>70</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="120">
@@ -2337,7 +2337,7 @@
         <v>70</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="120">
@@ -2357,7 +2357,7 @@
         <v>70</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="120">
@@ -2377,7 +2377,7 @@
         <v>71</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="120">
@@ -2417,7 +2417,7 @@
         <v>70</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="120">
@@ -2437,7 +2437,7 @@
         <v>70</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="120">
@@ -2457,7 +2457,7 @@
         <v>70</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="120">
@@ -2477,7 +2477,7 @@
         <v>70</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="120">
@@ -2497,7 +2497,7 @@
         <v>70</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="120">
@@ -2517,7 +2517,7 @@
         <v>72</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="120">
@@ -2537,7 +2537,7 @@
         <v>70</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="120">
@@ -2557,7 +2557,7 @@
         <v>70</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="120">
@@ -2577,7 +2577,7 @@
         <v>70</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="120">
@@ -2597,7 +2597,7 @@
         <v>70</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="120">
@@ -2617,7 +2617,7 @@
         <v>70</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="120">
@@ -2637,7 +2637,7 @@
         <v>70</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="30">
@@ -2708,7 +2708,7 @@
         <v>92</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="30">
@@ -2728,7 +2728,7 @@
         <v>123</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="30">
@@ -2748,7 +2748,7 @@
         <v>91</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="60">
@@ -2765,7 +2765,7 @@
         <v>94</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="30">
@@ -2876,7 +2876,7 @@
         <v>102</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>278</v>
+        <v>292</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="60">
@@ -2896,7 +2896,7 @@
         <v>132</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="60">
@@ -2916,7 +2916,7 @@
         <v>143</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="45">
@@ -2930,13 +2930,13 @@
         <v>111</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E83" s="1" t="s">
         <v>112</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="30">
@@ -2953,7 +2953,7 @@
         <v>117</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="85" spans="1:6">

</xml_diff>